<commit_message>
v3.0.0: Mitarbeiter-Dokumente Widget, Status-Verlauf editierbar, Dispo-Zeiten Popup, Markdowns 02.03
</commit_message>
<xml_diff>
--- a/Daten/Sonderaufgaben/Sonderaufgaben_2026_02_26.xlsx
+++ b/Daten/Sonderaufgaben/Sonderaufgaben_2026_02_26.xlsx
@@ -1290,13 +1290,13 @@
       <c r="B3" s="59" t="n"/>
       <c r="C3" s="55" t="inlineStr">
         <is>
-          <t>Yavgaan</t>
+          <t>Joisten</t>
         </is>
       </c>
       <c r="D3" s="59" t="n"/>
       <c r="E3" s="55" t="inlineStr">
         <is>
-          <t>Timera</t>
+          <t>Chugh</t>
         </is>
       </c>
       <c r="F3" s="59" t="n"/>
@@ -1311,7 +1311,7 @@
       <c r="B4" s="60" t="n"/>
       <c r="C4" s="55" t="inlineStr">
         <is>
-          <t>Kalbfleisch</t>
+          <t>Pieper</t>
         </is>
       </c>
       <c r="D4" s="59" t="n"/>
@@ -1328,7 +1328,7 @@
       <c r="B5" s="63" t="n"/>
       <c r="C5" s="55" t="inlineStr">
         <is>
-          <t>Campolo</t>
+          <t>Heim</t>
         </is>
       </c>
       <c r="D5" s="59" t="n"/>
@@ -1345,13 +1345,13 @@
       <c r="B6" s="60" t="n"/>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>Üzülmez</t>
+          <t>Christoffers</t>
         </is>
       </c>
       <c r="D6" s="60" t="n"/>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>Su</t>
+          <t>Adrovic</t>
         </is>
       </c>
       <c r="F6" s="60" t="n"/>
@@ -1366,13 +1366,13 @@
       <c r="B7" s="60" t="n"/>
       <c r="C7" s="16" t="inlineStr">
         <is>
-          <t>Bedl</t>
+          <t>Lemper</t>
         </is>
       </c>
       <c r="D7" s="60" t="n"/>
       <c r="E7" s="32" t="inlineStr">
         <is>
-          <t>Delgado</t>
+          <t>Idic</t>
         </is>
       </c>
       <c r="F7" s="64" t="n"/>
@@ -1393,7 +1393,7 @@
       <c r="D8" s="60" t="n"/>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>a.D</t>
+          <t>a.D.</t>
         </is>
       </c>
       <c r="F8" s="60" t="n"/>
@@ -1408,13 +1408,13 @@
       <c r="B9" s="60" t="n"/>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>Etz</t>
+          <t>Lemper</t>
         </is>
       </c>
       <c r="D9" s="60" t="n"/>
       <c r="E9" s="32" t="inlineStr">
         <is>
-          <t>Moeeni Mahvelati</t>
+          <t>Parso</t>
         </is>
       </c>
       <c r="F9" s="64" t="n"/>
@@ -1433,13 +1433,13 @@
       <c r="B10" s="60" t="n"/>
       <c r="C10" s="16" t="inlineStr">
         <is>
-          <t>Idic</t>
+          <t>Christoffers</t>
         </is>
       </c>
       <c r="D10" s="60" t="n"/>
       <c r="E10" s="32" t="inlineStr">
         <is>
-          <t>Rivola</t>
+          <t>Rasch</t>
         </is>
       </c>
       <c r="F10" s="64" t="n"/>

</xml_diff>